<commit_message>
feat: reclasificar ingreso Viaje Argentina de Febrero a AFP
</commit_message>
<xml_diff>
--- a/Finanzas Personales.xlsx
+++ b/Finanzas Personales.xlsx
@@ -170,10 +170,10 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ï¼­ï¼³ ï¼°ã´ã·ãã¯"/>
-        <a:font script="Hang" typeface="ë§ì ê³ ë"/>
-        <a:font script="Hans" typeface="å®ä½"/>
-        <a:font script="Hant" typeface="æ°ç´°æé«"/>
+        <a:font script="Jpan" typeface="Ã¯Â¼Â­Ã¯Â¼Â³ Ã¯Â¼Â°Ã£ÂÂ´Ã£ÂÂ·Ã£ÂÂÃ£ÂÂ¯"/>
+        <a:font script="Hang" typeface="Ã«Â§ÂÃ¬ÂÂ ÃªÂ³Â Ã«ÂÂ"/>
+        <a:font script="Hans" typeface="Ã¥Â®ÂÃ¤Â½Â"/>
+        <a:font script="Hant" typeface="Ã¦ÂÂ°Ã§Â´Â°Ã¦ÂÂÃ©Â«Â"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -205,10 +205,10 @@
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ï¼­ï¼³ ï¼°ã´ã·ãã¯"/>
-        <a:font script="Hang" typeface="ë§ì ê³ ë"/>
-        <a:font script="Hans" typeface="å®ä½"/>
-        <a:font script="Hant" typeface="æ°ç´°æé«"/>
+        <a:font script="Jpan" typeface="Ã¯Â¼Â­Ã¯Â¼Â³ Ã¯Â¼Â°Ã£ÂÂ´Ã£ÂÂ·Ã£ÂÂÃ£ÂÂ¯"/>
+        <a:font script="Hang" typeface="Ã«Â§ÂÃ¬ÂÂ ÃªÂ³Â Ã«ÂÂ"/>
+        <a:font script="Hans" typeface="Ã¥Â®ÂÃ¤Â½Â"/>
+        <a:font script="Hant" typeface="Ã¦ÂÂ°Ã§Â´Â°Ã¦ÂÂÃ©Â«Â"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -6348,10 +6348,10 @@
         <v>46059</v>
       </c>
       <c r="C119" t="str">
-        <v>Otro Ing</v>
+        <v>Sueldo</v>
       </c>
       <c r="D119" t="str">
-        <v>Viaje Argentina</v>
+        <v>AFP</v>
       </c>
       <c r="E119">
         <v>600</v>
@@ -31822,6 +31822,24 @@
       </c>
       <c r="G740" t="str">
         <v>Marzo</v>
+      </c>
+      <c r="H740" t="str">
+        <v/>
+      </c>
+      <c r="I740" t="str">
+        <v/>
+      </c>
+      <c r="J740" t="str">
+        <v/>
+      </c>
+      <c r="K740" t="str">
+        <v/>
+      </c>
+      <c r="L740" t="str">
+        <v/>
+      </c>
+      <c r="M740" t="str">
+        <v/>
       </c>
     </row>
   </sheetData>
@@ -34557,10 +34575,10 @@
         <v>46059</v>
       </c>
       <c r="C119" t="str">
-        <v>Otro Ing</v>
+        <v>Sueldo</v>
       </c>
       <c r="D119" t="str">
-        <v>Viaje Argentina</v>
+        <v>AFP</v>
       </c>
       <c r="E119">
         <v>600</v>

</xml_diff>